<commit_message>
test(app): localize privatbank fixtures and expand csv/mcc/picker flows
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/app-tests/fixtures/privatbank/privatbank-statement-001.xlsx
+++ b/tests/app-tests/fixtures/privatbank/privatbank-statement-001.xlsx
@@ -468,7 +468,7 @@
         <v>10.04.2026 10:15:00</v>
       </c>
       <c r="B3" t="str">
-        <v>Groceries</v>
+        <v>Супермаркети</v>
       </c>
       <c r="C3" t="str">
         <v>4149 0000 0000 1234</v>
@@ -500,7 +500,7 @@
         <v>11.04.2026 09:30:00</v>
       </c>
       <c r="B4" t="str">
-        <v>Salary</v>
+        <v>Зарахування</v>
       </c>
       <c r="C4" t="str">
         <v>4149 0000 0000 1234</v>

</xml_diff>

<commit_message>
feat: capture bank fees as a categorized split on sync and import (#502)
</commit_message>
<xml_diff>
--- a/tests/app-tests/fixtures/privatbank/privatbank-statement-001.xlsx
+++ b/tests/app-tests/fixtures/privatbank/privatbank-statement-001.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -524,6 +524,38 @@
         <v>2050</v>
       </c>
       <c r="J4" t="str">
+        <v>UAH</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>13.04.2026 18:00:00</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Зняття готівки</v>
+      </c>
+      <c r="C5" t="str">
+        <v>4149 0000 0000 1234</v>
+      </c>
+      <c r="D5" t="str">
+        <v>E2E Privatbank ATM</v>
+      </c>
+      <c r="E5">
+        <v>-303</v>
+      </c>
+      <c r="F5" t="str">
+        <v>UAH</v>
+      </c>
+      <c r="G5">
+        <v>-300</v>
+      </c>
+      <c r="H5" t="str">
+        <v>UAH</v>
+      </c>
+      <c r="I5">
+        <v>1747</v>
+      </c>
+      <c r="J5" t="str">
         <v>UAH</v>
       </c>
     </row>

</xml_diff>